<commit_message>
Reflect interviewer observation on candidate's ambition in evaluation form
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012mUmWTxBUioRfF9zJw7DFm
</commit_message>
<xml_diff>
--- a/interview-prep/(양식)_1차_역량인터뷰_가이드_및_평가표_김중환_260729.xlsx
+++ b/interview-prep/(양식)_1차_역량인터뷰_가이드_및_평가표_김중환_260729.xlsx
@@ -2673,7 +2673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W113"/>
+  <dimension ref="B1:W113"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10" defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col width="1.28515625" customWidth="1" style="58" min="1" max="1"/>
@@ -3897,7 +3897,7 @@
       <c r="I54" s="288" t="n"/>
       <c r="J54" s="311" t="inlineStr">
         <is>
-          <t>시스템 정비가 진행 중인 당사 상황과 부합하는 성향. 스스로 일을 찾아서 하는 태도가 확인됨.</t>
+          <t>시스템 정비가 진행 중인 당사 상황과 부합하는 성향. 스스로 일을 찾아서 하는 태도가 확인됨. 특히 조직 안에서 중요한 일을 맡아 기여하고자 하는 열망이 뚜렷한 점을 긍정적으로 평가함.</t>
         </is>
       </c>
       <c r="K54" s="292" t="n"/>
@@ -4267,7 +4267,7 @@
       <c r="F71" s="314" t="n"/>
       <c r="G71" s="317" t="inlineStr">
         <is>
-          <t>불리한 사실까지 선제적으로 공개하는 정직성, 역할 경계에 얽매이지 않고 스스로 일을 찾아 하는 성향, 높은 수준의 사전 조사에 기반한 지원 진정성이 확인되어 당사가 추구하는 핵심가치 및 업무 문화와의 적합도가 양호한 것으로 판단됨. PASS 의견으로 제시함.</t>
+          <t>불리한 사실까지 선제적으로 공개하는 정직성, 역할 경계에 얽매이지 않고 스스로 일을 찾아 하는 성향, 높은 수준의 사전 조사에 기반한 지원 진정성이 확인됨. 조직 안에서 중요한 일을 맡아 기여하고자 하는 열망이 뚜렷하여 상장 준비·내부 시스템 셋업 등 할 일이 많은 당사 상황과 잘 맞을 것으로 판단됨. PASS 의견으로 제시함.</t>
         </is>
       </c>
       <c r="H71" s="316" t="n"/>
@@ -4380,7 +4380,6 @@
       <c r="K79" s="63" t="n"/>
       <c r="L79" s="64" t="n"/>
     </row>
-    <row r="80"/>
     <row r="81" hidden="1" ht="18" customHeight="1" s="277">
       <c r="B81" s="93" t="inlineStr">
         <is>
@@ -5055,8 +5054,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14" ht="16.5" customHeight="1" s="277">
       <c r="C14" s="156" t="inlineStr">
         <is>
@@ -5104,8 +5101,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20" ht="16.5" customHeight="1" s="277">
       <c r="C20" s="156" t="inlineStr">
         <is>
@@ -5173,7 +5168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="B1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.28515625" defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col width="1.7109375" customWidth="1" style="4" min="1" max="1"/>

</xml_diff>